<commit_message>
Finalizando projeto, fiz os arquivos pdfs em ingles e portugues
</commit_message>
<xml_diff>
--- a/data/resultados_experimento.xlsx
+++ b/data/resultados_experimento.xlsx
@@ -589,35 +589,35 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-06-25T06:38:38.483281</t>
+          <t>2025-06-29T21:31:27.695655</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.05946581659882213</v>
+        <v>0.0642716523001127</v>
       </c>
       <c r="F2" t="n">
-        <v>0.001860439990734883</v>
+        <v>0.002986806940023528</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05827353199856589</v>
+        <v>0.05936170800032414</v>
       </c>
       <c r="H2" t="n">
-        <v>0.06438373799755936</v>
+        <v>0.06844271099998878</v>
       </c>
       <c r="I2" t="n">
-        <v>0.05877141199744074</v>
+        <v>0.06470139950010889</v>
       </c>
       <c r="J2" t="n">
-        <v>0.05867352774839674</v>
+        <v>0.06296408149989929</v>
       </c>
       <c r="K2" t="n">
-        <v>0.05909573875032947</v>
+        <v>0.06580232025009991</v>
       </c>
       <c r="L2" t="n">
-        <v>0.05813493800327305</v>
+        <v>0.06213501932871297</v>
       </c>
       <c r="M2" t="n">
-        <v>0.06079669519437121</v>
+        <v>0.06640828527151243</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -632,20 +632,20 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>168303.452328378</v>
+        <v>155896.6117900158</v>
       </c>
       <c r="S2" t="n">
-        <v>4959.7539915788</v>
+        <v>7348.646558730344</v>
       </c>
       <c r="T2" t="n">
-        <v>155318.7235009418</v>
+        <v>146107.5964685508</v>
       </c>
       <c r="U2" t="n">
-        <v>171604.4944769454</v>
+        <v>168458.7646963493</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>[0.05830308700387832, 0.05875803999515483, 0.05892295599915087, 0.05867070199747104, 0.05868200500117382, 0.06072598899481818, 0.05915333300072234, 0.05878478399972664, 0.06438373799755936, 0.058273531998565886]</t>
+          <t>[0.06287675299972761, 0.06603549300007217, 0.06510280200018315, 0.06322606700041433, 0.06844271099998878, 0.06452724300015689, 0.068101150000075, 0.06016704000012396, 0.0648755560000609, 0.05936170800032414]</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>[171517.504713512, 170189.47536072673, 169713.14202471628, 170442.82170734965, 170409.99195238762, 164674.13977981175, 169052.18172368896, 170112.04804369956, 155318.72350094176, 171604.4944769454]</t>
+          <t>[159041.29146177953, 151433.71459328805, 153603.21971966533, 158162.61352986685, 146107.59646855076, 154973.30329107176, 146840.3984365754, 166203.95485600416, 154141.26084700704, 168458.7646963493]</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -694,35 +694,35 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-06-25T06:38:39.919628</t>
+          <t>2025-06-29T21:31:29.215455</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.04849277650064323</v>
+        <v>0.05179314290003276</v>
       </c>
       <c r="F3" t="n">
-        <v>0.001860429118280827</v>
+        <v>0.006735991211896062</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04693179200694431</v>
+        <v>0.04704201300000932</v>
       </c>
       <c r="H3" t="n">
-        <v>0.05305616799887503</v>
+        <v>0.06835226499970304</v>
       </c>
       <c r="I3" t="n">
-        <v>0.04788758949871408</v>
+        <v>0.04897329549999085</v>
       </c>
       <c r="J3" t="n">
-        <v>0.04740723425129545</v>
+        <v>0.04739303075018597</v>
       </c>
       <c r="K3" t="n">
-        <v>0.04849251724954229</v>
+        <v>0.05445494474997759</v>
       </c>
       <c r="L3" t="n">
-        <v>0.04716190568277924</v>
+        <v>0.04697450506792615</v>
       </c>
       <c r="M3" t="n">
-        <v>0.04982364731850722</v>
+        <v>0.05661178073213938</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -737,20 +737,20 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>206474.4225520033</v>
+        <v>195585.1689254989</v>
       </c>
       <c r="S3" t="n">
-        <v>7480.507757924442</v>
+        <v>21577.58799858037</v>
       </c>
       <c r="T3" t="n">
-        <v>188479.4996919497</v>
+        <v>146300.9309207741</v>
       </c>
       <c r="U3" t="n">
-        <v>213075.1793692502</v>
+        <v>212575.9371733947</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>[0.0479675419992418, 0.04716456599999219, 0.046931792006944306, 0.04783396400307538, 0.04790342100022826, 0.05026605400053086, 0.04866750899964245, 0.04787175799719989, 0.04726499100070214, 0.053056167998875026]</t>
+          <t>[0.04704201300000932, 0.047657956999955786, 0.04712196300033611, 0.0473047220002627, 0.0479407729999366, 0.05075450699996509, 0.05000581800004511, 0.05568842399998175, 0.06835226499970304, 0.056062987000132125]</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>[208474.30539922317, 212023.57719143765, 213075.17936925017, 209056.47709558572, 208753.3581359951, 198941.41680376165, 205475.89563446667, 208891.4303206688, 211573.08587769425, 188479.49969194975]</t>
+          <t>[212575.93717339475, 209828.54972170288, 212215.26785564245, 211395.38670039043, 208590.71254468977, 197026.8374394195, 199976.73070743447, 179570.5333662033, 146300.93092077412, 178370.802825337]</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="AC3" t="n">
-        <v>1.226281951457932</v>
+        <v>1.240929758291846</v>
       </c>
     </row>
     <row r="4">
@@ -799,35 +799,35 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2025-06-25T06:38:41.413969</t>
+          <t>2025-06-29T21:31:30.827376</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.05688670610106783</v>
+        <v>0.059959496700003</v>
       </c>
       <c r="F4" t="n">
-        <v>0.002615851715837612</v>
+        <v>0.00661040440914978</v>
       </c>
       <c r="G4" t="n">
-        <v>0.05505975699634291</v>
+        <v>0.05535168899996279</v>
       </c>
       <c r="H4" t="n">
-        <v>0.06221978700341424</v>
+        <v>0.07585036599994055</v>
       </c>
       <c r="I4" t="n">
-        <v>0.05554619300164632</v>
+        <v>0.05655928400005905</v>
       </c>
       <c r="J4" t="n">
-        <v>0.05525108775145782</v>
+        <v>0.05560156425008245</v>
       </c>
       <c r="K4" t="n">
-        <v>0.05756724325328832</v>
+        <v>0.06130843375001405</v>
       </c>
       <c r="L4" t="n">
-        <v>0.05501543851110195</v>
+        <v>0.05523069825454193</v>
       </c>
       <c r="M4" t="n">
-        <v>0.05875797369103371</v>
+        <v>0.06468829514546406</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -842,20 +842,20 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>176106.2972875453</v>
+        <v>168379.1153065919</v>
       </c>
       <c r="S4" t="n">
-        <v>7693.719577874511</v>
+        <v>16195.69289689577</v>
       </c>
       <c r="T4" t="n">
-        <v>160720.5759070062</v>
+        <v>131838.5200673631</v>
       </c>
       <c r="U4" t="n">
-        <v>181620.8524251969</v>
+        <v>180662.9604384199</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>[0.055914750999363605, 0.05505975699634291, 0.05536678800126538, 0.058118074004596565, 0.06080419399950188, 0.055212521001521964, 0.06221978700341424, 0.05507880300137913, 0.05544265400385484, 0.05564973199943779]</t>
+          <t>[0.06588900199994896, 0.07585036599994055, 0.061285035999844695, 0.0613162330000705, 0.05704139799991026, 0.05535168899996279, 0.05607717000020784, 0.05556135799997719, 0.05550053199976901, 0.05572218300039822]</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>[178843.68295074435, 181620.85242519694, 180613.6920886842, 172063.51330928653, 164462.33955641155, 181118.3372649176, 160720.57590700625, 181558.0487424465, 180366.54593239198, 179695.38469836704]</t>
+          <t>[151770.39712952013, 131838.52006736313, 163171.96909250965, 163088.94905511403, 175311.27129836005, 180662.96043841992, 178325.68940199615, 179981.20204340768, 180178.45306494753, 179461.74147428028]</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -904,35 +904,35 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2025-06-25T06:38:42.941213</t>
+          <t>2025-06-29T21:31:32.306718</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.05737408799905097</v>
+        <v>0.05541215320008632</v>
       </c>
       <c r="F5" t="n">
-        <v>0.003278322904571118</v>
+        <v>0.0008975726045036777</v>
       </c>
       <c r="G5" t="n">
-        <v>0.05513511999743059</v>
+        <v>0.0548527680002735</v>
       </c>
       <c r="H5" t="n">
-        <v>0.06597674200020265</v>
+        <v>0.05792404800013173</v>
       </c>
       <c r="I5" t="n">
-        <v>0.05641957150146482</v>
+        <v>0.05517874600013783</v>
       </c>
       <c r="J5" t="n">
-        <v>0.05530199624809029</v>
+        <v>0.05503808524974829</v>
       </c>
       <c r="K5" t="n">
-        <v>0.05794338024861645</v>
+        <v>0.0552928245002704</v>
       </c>
       <c r="L5" t="n">
-        <v>0.05502891706920627</v>
+        <v>0.05477006843882867</v>
       </c>
       <c r="M5" t="n">
-        <v>0.05971925892889567</v>
+        <v>0.05605423796134397</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -947,20 +947,20 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>174759.4558026731</v>
+        <v>180506.877359197</v>
       </c>
       <c r="S5" t="n">
-        <v>9049.990222135866</v>
+        <v>2816.038377731491</v>
       </c>
       <c r="T5" t="n">
-        <v>151568.5633578161</v>
+        <v>172639.8679867342</v>
       </c>
       <c r="U5" t="n">
-        <v>181372.5988166167</v>
+        <v>182306.2055856532</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>[0.05595914000150515, 0.0586403689958388, 0.056975457999214996, 0.06597674200020265, 0.056880003001424484, 0.058266020998416934, 0.05525418699835427, 0.05544542399729835, 0.05520841600082349, 0.05513511999743059]</t>
+          <t>[0.054921275000197056, 0.0548527680002735, 0.055197532999955, 0.055300392000390275, 0.05515995900032067, 0.05500521599969943, 0.057924048000131734, 0.05527012199991077, 0.055136692999894876, 0.055353526000089914]</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>[178701.8170710098, 170530.98695046775, 175514.16611934526, 151568.56335781608, 175808.71083550336, 171626.61579845476, 180981.7598130228, 180357.53501474284, 181131.80424975132, 181372.5988166167]</t>
+          <t>[182078.80279480256, 182306.2055856532, 181167.51703392528, 180830.54456339887, 181290.92517893034, 181800.94047907463, 172639.86798673423, 180929.58072385192, 181367.4244122524, 180656.96483334695]</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="AC5" t="n">
-        <v>0.9915051913680754</v>
+        <v>1.082064010100759</v>
       </c>
     </row>
     <row r="6">
@@ -1009,73 +1009,73 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2025-06-25T06:38:51.264037</t>
+          <t>2025-06-29T21:31:40.955936</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.7149365504999878</v>
+        <v>0.7424729585999558</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01313972176666356</v>
+        <v>0.02113974497291606</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6998494830040727</v>
+        <v>0.7046222049998505</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7412023779979791</v>
+        <v>0.7689441210000041</v>
       </c>
       <c r="I6" t="n">
-        <v>0.7134550694972859</v>
+        <v>0.74634063350004</v>
       </c>
       <c r="J6" t="n">
-        <v>0.7049925172486837</v>
+        <v>0.7411172144998091</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7188240324976505</v>
+        <v>0.7519812880001382</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7055369597914397</v>
+        <v>0.7273504960427479</v>
       </c>
       <c r="M6" t="n">
-        <v>0.724336141208536</v>
+        <v>0.7575954211571636</v>
       </c>
       <c r="N6" t="n">
-        <v>1.558984375</v>
+        <v>3.285546875</v>
       </c>
       <c r="O6" t="n">
-        <v>0.7795564326000222</v>
+        <v>0.1964070890495204</v>
       </c>
       <c r="P6" t="n">
-        <v>1.28515625</v>
+        <v>2.7265625</v>
       </c>
       <c r="Q6" t="n">
-        <v>3.765625</v>
+        <v>3.34765625</v>
       </c>
       <c r="R6" t="n">
-        <v>139914.5077523285</v>
+        <v>134785.6581354807</v>
       </c>
       <c r="S6" t="n">
-        <v>2536.838948912026</v>
+        <v>3927.93679459333</v>
       </c>
       <c r="T6" t="n">
-        <v>134915.9190100071</v>
+        <v>130048.4616098645</v>
       </c>
       <c r="U6" t="n">
-        <v>142887.8672178973</v>
+        <v>141920.0236529889</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>[0.7114874539984157, 0.7313902220048476, 0.6998494830040727, 0.7045987829988007, 0.7194652179969125, 0.7061737199983327, 0.7169004759998643, 0.715422684996156, 0.7028750860044966, 0.7412023779979791]</t>
+          <t>[0.7077368860000206, 0.7046222049998505, 0.7469167160002144, 0.7641639669996039, 0.7517529910001031, 0.7408490479997454, 0.7689441210000041, 0.7520573870001499, 0.7419217140000001, 0.7457645509998656]</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>[3.765625, 1.54296875, 1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625]</t>
+          <t>[2.7265625, 3.34765625, 3.34765625, 3.34765625, 3.34765625, 3.34765625, 3.34765625, 3.34765625, 3.34765625, 3.34765625]</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>[140550.61609030518, 136725.91865650783, 142887.8672178973, 141924.74130369056, 138992.12567692067, 141608.2150440774, 139489.3759284084, 139777.5078945635, 142272.79070090735, 134915.91901000708]</t>
+          <t>[141295.44747226455, 141920.02365298892, 133883.73543908112, 130861.96721972869, 133022.41719978245, 134980.2638877581, 130048.46160986446, 132968.5762397545, 134785.11022525484, 134090.57840832934]</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -1114,73 +1114,73 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2025-06-25T06:39:03.744452</t>
+          <t>2025-06-29T21:31:54.335485</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1.125886663700658</v>
+        <v>1.210067964900009</v>
       </c>
       <c r="F7" t="n">
-        <v>0.005601899508837191</v>
+        <v>0.0603754622000333</v>
       </c>
       <c r="G7" t="n">
-        <v>1.119707912002923</v>
+        <v>1.146663179999905</v>
       </c>
       <c r="H7" t="n">
-        <v>1.135155918003875</v>
+        <v>1.33491241999991</v>
       </c>
       <c r="I7" t="n">
-        <v>1.125353981999069</v>
+        <v>1.196193957499872</v>
       </c>
       <c r="J7" t="n">
-        <v>1.120632753252721</v>
+        <v>1.16844721450002</v>
       </c>
       <c r="K7" t="n">
-        <v>1.129864422249739</v>
+        <v>1.225062132000176</v>
       </c>
       <c r="L7" t="n">
-        <v>1.121879306200358</v>
+        <v>1.166877961062977</v>
       </c>
       <c r="M7" t="n">
-        <v>1.129894021200957</v>
+        <v>1.25325796873704</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>0.063671875</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>0.2013481478935335</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>0.63671875</v>
       </c>
       <c r="R7" t="n">
-        <v>88820.86248949837</v>
+        <v>82817.52601386004</v>
       </c>
       <c r="S7" t="n">
-        <v>441.229373328749</v>
+        <v>3957.581777393328</v>
       </c>
       <c r="T7" t="n">
-        <v>88093.62521392295</v>
+        <v>74911.28144571969</v>
       </c>
       <c r="U7" t="n">
-        <v>89309.0054361775</v>
+        <v>87209.56750351771</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>[1.1351559180038748, 1.1259120059985435, 1.1204751640034374, 1.1286890979972668, 1.1326117710050312, 1.1211055210005725, 1.1302561970005627, 1.119707912002923, 1.1201570919947699, 1.124795957999595]</t>
+          <t>[1.154461855000136, 1.2284966760003044, 1.3349124199999096, 1.2884339110000838, 1.1999294229999578, 1.214758499999789, 1.1739533590002793, 1.1666118329999335, 1.192458491999787, 1.146663179999905]</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>[0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0]</t>
+          <t>[0.63671875, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0]</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>[88093.62521392295, 88816.88752516008, 89247.85056609538, 88598.35731331052, 88291.50690466892, 89197.6697347376, 88475.51578604635, 89309.0054361775, 89273.19276434748, 88905.0136505167]</t>
+          <t>[86620.44533293672, 81400.30164800806, 74911.2814457197, 77613.604505628, 83338.23480216763, 82320.8892961172, 85182.25978343676, 85718.31449956303, 83860.36132150574, 87209.56750351771]</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="AC7" t="n">
-        <v>0.63499868463676</v>
+        <v>0.6135795510141518</v>
       </c>
     </row>
     <row r="8">
@@ -1219,73 +1219,73 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2025-06-25T06:39:11.634842</t>
+          <t>2025-06-29T21:32:02.537335</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.6780599705984059</v>
+        <v>0.7039190375000089</v>
       </c>
       <c r="F8" t="n">
-        <v>0.01232589718933624</v>
+        <v>0.01365855955939503</v>
       </c>
       <c r="G8" t="n">
-        <v>0.664658479996433</v>
+        <v>0.6797443229997953</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7069873859945801</v>
+        <v>0.7271815169997353</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6737814385014644</v>
+        <v>0.7050614390000192</v>
       </c>
       <c r="J8" t="n">
-        <v>0.6707823382457718</v>
+        <v>0.6997516280001719</v>
       </c>
       <c r="K8" t="n">
-        <v>0.684062688749691</v>
+        <v>0.7120660575000102</v>
       </c>
       <c r="L8" t="n">
-        <v>0.669242554921512</v>
+        <v>0.6941482925933427</v>
       </c>
       <c r="M8" t="n">
-        <v>0.6868773862752999</v>
+        <v>0.7136897824066752</v>
       </c>
       <c r="N8" t="n">
-        <v>1.28515625</v>
+        <v>2.5484375</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>0.6482445119440851</v>
       </c>
       <c r="P8" t="n">
-        <v>1.28515625</v>
+        <v>2.31640625</v>
       </c>
       <c r="Q8" t="n">
-        <v>1.28515625</v>
+        <v>4.37890625</v>
       </c>
       <c r="R8" t="n">
-        <v>147522.5147444713</v>
+        <v>142110.1911207669</v>
       </c>
       <c r="S8" t="n">
-        <v>2624.809355217112</v>
+        <v>2772.226822203612</v>
       </c>
       <c r="T8" t="n">
-        <v>141445.2393083667</v>
+        <v>137517.2466052054</v>
       </c>
       <c r="U8" t="n">
-        <v>150453.2071877525</v>
+        <v>147114.1377962345</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>[0.6727143680036534, 0.664658479996433, 0.6704657519949251, 0.7069873859945801, 0.6851861309987726, 0.6806923620024463, 0.6748485089992755, 0.6853952940000454, 0.671732096998312, 0.6679193269956158]</t>
+          <t>[0.7021027790001426, 0.7038913890000913, 0.7135879550000936, 0.7271815169997353, 0.6861508380002306, 0.7138318090001121, 0.706231488999947, 0.6989679110001816, 0.7075003649997598, 0.6797443229997953]</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>[1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625, 1.28515625]</t>
+          <t>[2.57421875, 4.37890625, 2.31640625, 2.31640625, 2.31640625, 2.31640625, 2.31640625, 2.31640625, 2.31640625, 2.31640625]</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>[148651.50018537574, 150453.20718775253, 149150.0493536871, 141445.2393083667, 145945.74448585729, 146909.24356169082, 148181.4046656023, 145901.20602723802, 148868.87264559473, 149718.6800235478]</t>
+          <t>[142429.28954420175, 142067.37227181369, 140136.89454719968, 137517.24660520544, 145740.5492521841, 140089.02200656108, 141596.6316393002, 143068.084280015, 141342.68326495343, 147114.13779623448]</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -1324,35 +1324,35 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-06-25T06:39:20.795399</t>
+          <t>2025-06-29T21:32:11.936524</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.8049381130993425</v>
+        <v>0.8228220055000748</v>
       </c>
       <c r="F9" t="n">
-        <v>0.01783837122805005</v>
+        <v>0.02034976296448907</v>
       </c>
       <c r="G9" t="n">
-        <v>0.7856258259998867</v>
+        <v>0.7923847860001842</v>
       </c>
       <c r="H9" t="n">
-        <v>0.8354895779993967</v>
+        <v>0.8524907999999414</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7960413754990441</v>
+        <v>0.8232278159998714</v>
       </c>
       <c r="J9" t="n">
-        <v>0.7909815362490917</v>
+        <v>0.8066717545002575</v>
       </c>
       <c r="K9" t="n">
-        <v>0.819535676500891</v>
+        <v>0.8387033682499805</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7921773110497732</v>
+        <v>0.8082646620282018</v>
       </c>
       <c r="M9" t="n">
-        <v>0.8176989151489118</v>
+        <v>0.8373793489719478</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
@@ -1367,20 +1367,20 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>124287.4826278376</v>
+        <v>121600.0058892416</v>
       </c>
       <c r="S9" t="n">
-        <v>2724.208963191619</v>
+        <v>3012.315990646543</v>
       </c>
       <c r="T9" t="n">
-        <v>119690.3021093965</v>
+        <v>117303.3186985794</v>
       </c>
       <c r="U9" t="n">
-        <v>127287.0578977306</v>
+        <v>126201.3125022024</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>[0.8157998349997797, 0.793910833002883, 0.8354895779993967, 0.8207809570012614, 0.7976964659974328, 0.826054134995502, 0.790005103997828, 0.7896321119987988, 0.7943862850006553, 0.7856258259998867]</t>
+          <t>[0.8046036650002861, 0.8018237240003145, 0.8128760230001717, 0.812883771000088, 0.7923847860001842, 0.8524907999999414, 0.8350030609999521, 0.8335718609996547, 0.8399368039999899, 0.8426455600001646]</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>[122579.08828827724, 125958.72967466721, 119690.30210939652, 121835.18531588728, 125360.96656133591, 121057.44135103752, 126581.46066898694, 126641.25290810376, 125883.34150295345, 127287.05789773058]</t>
+          <t>[124284.79306015147, 124715.6912508126, 123019.98972846918, 123018.81716370146, 126201.31250220237, 117303.31869857936, 119760.0400173931, 119965.66184476975, 119056.57607069353, 118673.85855564286]</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="AC9" t="n">
-        <v>0.8423752827252724</v>
+        <v>0.8554936946201361</v>
       </c>
     </row>
   </sheetData>

</xml_diff>